<commit_message>
Daily rebuild 2026-09-10 (run 4)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="combined" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="benchmark-scout" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="news-scout" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="editor" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="verifier" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="commentator" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rebuild" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="combined" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="benchmark-scout" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="news-scout" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="editor" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="verifier" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="commentator" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="rebuild" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -654,6 +654,117 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>4 considered under 10; 3 picked</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>AA_API_KEY not set</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>AA_API_KEY not set</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>AA_API_KEY not set</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1202,6 +1313,117 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>AA_API_KEY not set</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>AA_API_KEY not set</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>AA_API_KEY not set</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-10 (run 5)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -765,6 +765,43 @@
       <c r="G9" t="inlineStr">
         <is>
           <t>AA_API_KEY not set</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>13:08</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>numbers carried forward (--no-fetch)</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1424,6 +1461,43 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>13:08</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>numbers carried forward (--no-fetch)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-10 (run 6)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -802,6 +802,43 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>numbers carried forward (--no-fetch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; tau carried forward; omni carried forward; nohalluc carried forward; gdppdf</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1498,6 +1535,43 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; tau carried forward; omni carried forward; nohalluc carried forward; gdppdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-10 (run 8)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -839,6 +839,80 @@
       <c r="G11" t="inlineStr">
         <is>
           <t>gdpval carried forward; tau carried forward; omni carried forward; nohalluc carried forward; gdppdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>commentator</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>first live run status partial data</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1327,6 +1401,43 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>commentator</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>first live run status partial data</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1338,7 +1449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1572,6 +1683,43 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-10 (run 9)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -913,6 +913,43 @@
       <c r="G13" t="inlineStr">
         <is>
           <t>first live run status partial data</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1720,6 +1757,43 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-10 (run 10)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -948,6 +948,43 @@
         </is>
       </c>
       <c r="G14" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
         </is>
@@ -1486,7 +1523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1794,6 +1831,43 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-10 (run 11)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -985,6 +985,43 @@
         </is>
       </c>
       <c r="G15" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
         </is>
@@ -1523,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1868,6 +1905,43 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-11 (run 12)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1024,6 +1024,80 @@
       <c r="G16" t="inlineStr">
         <is>
           <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>commentator</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>data/2026-09-11.json missing on main after 10m retry</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1549,6 +1623,43 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>commentator</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>data/2026-09-11.json missing on main after 10m retry</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1560,7 +1671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1942,6 +2053,43 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-11 (run 13)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,43 @@
       <c r="G18" t="inlineStr">
         <is>
           <t>data/2026-09-11.json missing on main after 10m retry</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2090,6 +2127,43 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-11 (run 14)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1133,6 +1133,43 @@
         </is>
       </c>
       <c r="G19" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
         <is>
           <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
         </is>
@@ -1708,7 +1745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2164,6 +2201,43 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-12 (run 16)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1172,6 +1172,80 @@
       <c r="G20" t="inlineStr">
         <is>
           <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>commentator</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>data/2026-09-12.json missing on main after 10m retry</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1734,6 +1808,43 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>commentator</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>data/2026-09-12.json missing on main after 10m retry</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1745,7 +1856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2238,6 +2349,43 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-12 (run 15)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1246,6 +1246,43 @@
       <c r="G22" t="inlineStr">
         <is>
           <t>data/2026-09-12.json missing on main after 10m retry</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2386,6 +2423,43 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-12 (run 17)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1281,6 +1281,43 @@
         </is>
       </c>
       <c r="G23" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
         </is>
@@ -1893,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2460,6 +2497,43 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-13 (run 18)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1318,6 +1318,43 @@
         </is>
       </c>
       <c r="G24" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
         </is>
@@ -1930,7 +1967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2534,6 +2571,43 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily rebuild 2026-09-13 (run 19)
</commit_message>
<xml_diff>
--- a/log/run-log.xlsx
+++ b/log/run-log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1357,6 +1357,43 @@
       <c r="G25" t="inlineStr">
         <is>
           <t>gdpval carried forward; omni carried forward; nohalluc carried forward; gdppdf carried forward; web</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>cost missing or carried forward; gdppdf carried forward</t>
         </is>
       </c>
     </row>
@@ -1967,7 +2004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2608,6 +2645,43 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>rebuild</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>cost missing or carried forward; gdppdf carried forward</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>